<commit_message>
refactor: migrate schedule and calendar logic to edustack_schedule
</commit_message>
<xml_diff>
--- a/data/fall26_generated_schedule.xlsx
+++ b/data/fall26_generated_schedule.xlsx
@@ -931,253 +931,9 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E13"/>
+  <dimension ref="A1:A1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>Section</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>Date</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>Assignments</t>
-        </is>
-      </c>
-      <c r="D1" t="inlineStr">
-        <is>
-          <t>Project Milestones</t>
-        </is>
-      </c>
-      <c r="E1" t="inlineStr">
-        <is>
-          <t>Participation</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>O1</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>17-Sep (Thu)</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>A1 (Due: Sep 26)</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr"/>
-      <c r="E2" t="inlineStr"/>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>O1</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>17-Sep (Thu)</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr"/>
-      <c r="D3" t="inlineStr"/>
-      <c r="E3" t="inlineStr"/>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>O1</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>24-Sep (Thu)</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>A2 (Due: Oct 03)</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr"/>
-      <c r="E4" t="inlineStr"/>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>O1</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>24-Sep (Thu)</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr"/>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>Ungraded Milestone 1</t>
-        </is>
-      </c>
-      <c r="E5" t="inlineStr"/>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>O1</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>01-Oct (Thu)</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>A3 (Due: Oct 10)</t>
-        </is>
-      </c>
-      <c r="D6" t="inlineStr"/>
-      <c r="E6" t="inlineStr"/>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>O1</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>01-Oct (Thu)</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr"/>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>Ungraded Milestone 2</t>
-        </is>
-      </c>
-      <c r="E7" t="inlineStr"/>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>O1</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>08-Oct (Thu)</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>A4 (Due: Oct 17)</t>
-        </is>
-      </c>
-      <c r="D8" t="inlineStr"/>
-      <c r="E8" t="inlineStr"/>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>O1</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>08-Oct (Thu)</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr"/>
-      <c r="D9" t="inlineStr"/>
-      <c r="E9" t="inlineStr"/>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>O1</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>15-Oct (Thu)</t>
-        </is>
-      </c>
-      <c r="C10" t="inlineStr"/>
-      <c r="D10" t="inlineStr"/>
-      <c r="E10" t="inlineStr"/>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>O1</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>15-Oct (Thu)</t>
-        </is>
-      </c>
-      <c r="C11" t="inlineStr"/>
-      <c r="D11" t="inlineStr">
-        <is>
-          <t>Ungraded Milestone 3</t>
-        </is>
-      </c>
-      <c r="E11" t="inlineStr">
-        <is>
-          <t>Participation 1 + Participation 2</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>O1</t>
-        </is>
-      </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>22-Oct (Thu)</t>
-        </is>
-      </c>
-      <c r="C12" t="inlineStr"/>
-      <c r="D12" t="inlineStr"/>
-      <c r="E12" t="inlineStr"/>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>O1</t>
-        </is>
-      </c>
-      <c r="B13" t="inlineStr">
-        <is>
-          <t>22-Oct (Thu)</t>
-        </is>
-      </c>
-      <c r="C13" t="inlineStr"/>
-      <c r="D13" t="inlineStr">
-        <is>
-          <t>Final Project Report + Presentation</t>
-        </is>
-      </c>
-      <c r="E13" t="inlineStr"/>
-    </row>
-  </sheetData>
+  <sheetData/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -1188,261 +944,9 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E13"/>
+  <dimension ref="A1:A1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>Section</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>Date</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>Assignments</t>
-        </is>
-      </c>
-      <c r="D1" t="inlineStr">
-        <is>
-          <t>Project Milestones</t>
-        </is>
-      </c>
-      <c r="E1" t="inlineStr">
-        <is>
-          <t>Participation</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>A1</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>14-Sep (Mon)</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr"/>
-      <c r="D2" t="inlineStr"/>
-      <c r="E2" t="inlineStr"/>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>A1</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>21-Sep (Mon)</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>A1 (Due: Sep 22)</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr"/>
-      <c r="E3" t="inlineStr"/>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>A1</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>28-Sep (Mon)</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr"/>
-      <c r="D4" t="inlineStr"/>
-      <c r="E4" t="inlineStr"/>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>A1</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>05-Oct (Mon)</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>A2 (Due: Oct 06)</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>Ungraded Milestone 1</t>
-        </is>
-      </c>
-      <c r="E5" t="inlineStr"/>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>A1</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>13-Oct (Tue)</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr"/>
-      <c r="D6" t="inlineStr"/>
-      <c r="E6" t="inlineStr"/>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>A1</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>19-Oct (Mon)</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr"/>
-      <c r="D7" t="inlineStr"/>
-      <c r="E7" t="inlineStr"/>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>A1</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>26-Oct (Mon)</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>A3 (Due: Oct 27)</t>
-        </is>
-      </c>
-      <c r="D8" t="inlineStr">
-        <is>
-          <t>Ungraded Milestone 2</t>
-        </is>
-      </c>
-      <c r="E8" t="inlineStr"/>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>A1</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>02-Nov (Mon)</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr"/>
-      <c r="D9" t="inlineStr"/>
-      <c r="E9" t="inlineStr"/>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>A1</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>09-Nov (Mon)</t>
-        </is>
-      </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>A4 (Due: Nov 10)</t>
-        </is>
-      </c>
-      <c r="D10" t="inlineStr">
-        <is>
-          <t>Ungraded Milestone 3</t>
-        </is>
-      </c>
-      <c r="E10" t="inlineStr"/>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>A1</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>16-Nov (Mon)</t>
-        </is>
-      </c>
-      <c r="C11" t="inlineStr"/>
-      <c r="D11" t="inlineStr"/>
-      <c r="E11" t="inlineStr"/>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>A1</t>
-        </is>
-      </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>23-Nov (Mon)</t>
-        </is>
-      </c>
-      <c r="C12" t="inlineStr">
-        <is>
-          <t>A5 (Due: Nov 24)</t>
-        </is>
-      </c>
-      <c r="D12" t="inlineStr">
-        <is>
-          <t>Presentation</t>
-        </is>
-      </c>
-      <c r="E12" t="inlineStr">
-        <is>
-          <t>Participation 1 + Participation 2</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>A1</t>
-        </is>
-      </c>
-      <c r="B13" t="inlineStr">
-        <is>
-          <t>30-Nov (Mon)</t>
-        </is>
-      </c>
-      <c r="C13" t="inlineStr"/>
-      <c r="D13" t="inlineStr">
-        <is>
-          <t>Final Project Report + Presentation</t>
-        </is>
-      </c>
-      <c r="E13" t="inlineStr"/>
-    </row>
-  </sheetData>
+  <sheetData/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>